<commit_message>
Update of latest hs file
</commit_message>
<xml_diff>
--- a/Harbour Survey/raw data/2026/hs-0923-26.xlsx
+++ b/Harbour Survey/raw data/2026/hs-0923-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\tech\Archived Harbour data\HS2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\POURFARAJV\Documents\GitHub\Environmental-data\Harbour Survey\raw data\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3696E3F-DF4A-4A95-85F3-433109580568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D838CA6-4453-4FE1-BD40-A31111FD630E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="397" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="96">
   <si>
     <t xml:space="preserve">Depth  </t>
   </si>
@@ -586,9 +586,6 @@
   </si>
   <si>
     <t>D.O.</t>
-  </si>
-  <si>
-    <t>23/9/2026</t>
   </si>
   <si>
     <t>Cloudy, Steady Wind, Small waves</t>
@@ -1889,7 +1886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr syncVertical="1" syncRef="B2" transitionEvaluation="1">
+  <sheetPr syncVertical="1" syncRef="B61" transitionEvaluation="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AK99"/>
@@ -1948,8 +1945,8 @@
       <c r="Z1" s="40"/>
     </row>
     <row r="2" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="151" t="s">
-        <v>92</v>
+      <c r="B2" s="151">
+        <v>46288</v>
       </c>
       <c r="C2" s="152"/>
       <c r="D2" s="152"/>
@@ -3121,7 +3118,7 @@
         <v>22</v>
       </c>
       <c r="J25" s="123" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K25" s="138"/>
       <c r="L25" s="138"/>
@@ -3190,7 +3187,7 @@
         <v>22</v>
       </c>
       <c r="C28" s="123" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D28" s="138"/>
       <c r="E28" s="138"/>
@@ -4214,7 +4211,7 @@
         <v>22</v>
       </c>
       <c r="C52" s="123" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D52" s="138"/>
       <c r="E52" s="138"/>
@@ -4225,7 +4222,7 @@
         <v>22</v>
       </c>
       <c r="J52" s="123" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K52" s="138"/>
       <c r="L52" s="138"/>
@@ -5337,7 +5334,6 @@
   <mergeCells count="10">
     <mergeCell ref="M33:N33"/>
     <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
     <mergeCell ref="F33:G33"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="M4:N4"/>
@@ -5345,6 +5341,7 @@
     <mergeCell ref="I3:O3"/>
     <mergeCell ref="I32:O32"/>
     <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B2:O2"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="C6:C25 J6:J23 J35:J50 C35:C50">
@@ -5364,18 +5361,6 @@
         <cfvo type="percentile" val="80"/>
         <cfvo type="max"/>
         <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F26 M23 F50 M50">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="75"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF0000"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
@@ -5405,10 +5390,24 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="M23 F26 F50 M50">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="75"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0.25" top="1" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="90" orientation="portrait" horizontalDpi="1200" r:id="rId1"/>
-  <headerFooter alignWithMargins="0"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
+  </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -5499,9 +5498,9 @@
       <c r="D2" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="108" t="str">
+      <c r="E2" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F2" s="109">
         <f>Report!$C$51</f>
@@ -5534,9 +5533,9 @@
         <f>IF(Report!G35&gt;=0,Report!G35,"")</f>
         <v>0.89644523040647905</v>
       </c>
-      <c r="N2" s="110" t="e">
+      <c r="N2" s="110">
         <f>E2+F2</f>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O2" t="str">
         <f>"River: Flow = " &amp;Report!H59</f>
@@ -5560,9 +5559,9 @@
       <c r="D3" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="108" t="str">
+      <c r="E3" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F3" s="109">
         <f>Report!$C$51</f>
@@ -5596,9 +5595,9 @@
         <f>IF(Report!G36&gt;=0,Report!G36,"")</f>
         <v>0.99053193023575359</v>
       </c>
-      <c r="N3" s="110" t="e">
+      <c r="N3" s="110">
         <f t="shared" ref="N3:N66" si="0">E3+F3</f>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O3" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5622,9 +5621,9 @@
       <c r="D4" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="108" t="str">
+      <c r="E4" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F4" s="109">
         <f>Report!$C$51</f>
@@ -5658,9 +5657,9 @@
         <f>IF(Report!G37&gt;=0,Report!G37,"")</f>
         <v>0.99043008476310901</v>
       </c>
-      <c r="N4" s="110" t="e">
+      <c r="N4" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O4" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5684,9 +5683,9 @@
       <c r="D5" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="108" t="str">
+      <c r="E5" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F5" s="109">
         <f>Report!$C$51</f>
@@ -5720,9 +5719,9 @@
         <f>IF(Report!G38&gt;=0,Report!G38,"")</f>
         <v>1.0088948546282019</v>
       </c>
-      <c r="N5" s="110" t="e">
+      <c r="N5" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O5" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5746,9 +5745,9 @@
       <c r="D6" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="108" t="str">
+      <c r="E6" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F6" s="109">
         <f>Report!$C$51</f>
@@ -5782,9 +5781,9 @@
         <f>IF(Report!G39&gt;=0,Report!G39,"")</f>
         <v>0.90606331995159528</v>
       </c>
-      <c r="N6" s="110" t="e">
+      <c r="N6" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O6" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5808,9 +5807,9 @@
       <c r="D7" t="s">
         <v>71</v>
       </c>
-      <c r="E7" s="108" t="str">
+      <c r="E7" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F7" s="109">
         <f>Report!$C$51</f>
@@ -5844,9 +5843,9 @@
         <f>IF(Report!G40&gt;=0,Report!G40,"")</f>
         <v>0.63748647724249763</v>
       </c>
-      <c r="N7" s="110" t="e">
+      <c r="N7" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O7" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5870,9 +5869,9 @@
       <c r="D8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="108" t="str">
+      <c r="E8" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F8" s="109">
         <f>Report!$C$51</f>
@@ -5906,9 +5905,9 @@
         <f>IF(Report!G41&gt;=0,Report!G41,"")</f>
         <v>0.37118772848558035</v>
       </c>
-      <c r="N8" s="110" t="e">
+      <c r="N8" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O8" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5932,9 +5931,9 @@
       <c r="D9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="108" t="str">
+      <c r="E9" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F9" s="109">
         <f>Report!$C$51</f>
@@ -5968,9 +5967,9 @@
         <f>IF(Report!G42&gt;=0,Report!G42,"")</f>
         <v>0.33527549974372117</v>
       </c>
-      <c r="N9" s="110" t="e">
+      <c r="N9" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O9" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -5994,9 +5993,9 @@
       <c r="D10" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="108" t="str">
+      <c r="E10" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F10" s="109">
         <f>Report!$C$51</f>
@@ -6030,9 +6029,9 @@
         <f>IF(Report!G43&gt;=0,Report!G43,"")</f>
         <v>0.32938211369600517</v>
       </c>
-      <c r="N10" s="110" t="e">
+      <c r="N10" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O10" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6056,9 +6055,9 @@
       <c r="D11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="108" t="str">
+      <c r="E11" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F11" s="109">
         <f>Report!$C$51</f>
@@ -6092,9 +6091,9 @@
         <f>IF(Report!G44&gt;=0,Report!G44,"")</f>
         <v>0.30792886258922009</v>
       </c>
-      <c r="N11" s="110" t="e">
+      <c r="N11" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O11" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6118,9 +6117,9 @@
       <c r="D12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="108" t="str">
+      <c r="E12" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F12" s="109">
         <f>Report!$C$51</f>
@@ -6154,9 +6153,9 @@
         <f>IF(Report!G45&gt;=0,Report!G45,"")</f>
         <v>0.29611748402494414</v>
       </c>
-      <c r="N12" s="110" t="e">
+      <c r="N12" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O12" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6180,9 +6179,9 @@
       <c r="D13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="108" t="str">
+      <c r="E13" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F13" s="109">
         <f>Report!$C$51</f>
@@ -6216,9 +6215,9 @@
         <f>IF(Report!G46&gt;=0,Report!G46,"")</f>
         <v>0.26323344287791273</v>
       </c>
-      <c r="N13" s="110" t="e">
+      <c r="N13" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O13" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6242,9 +6241,9 @@
       <c r="D14" t="s">
         <v>71</v>
       </c>
-      <c r="E14" s="108" t="str">
+      <c r="E14" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F14" s="109">
         <f>Report!$C$51</f>
@@ -6278,9 +6277,9 @@
         <f>IF(Report!G47&gt;=0,Report!G47,"")</f>
         <v/>
       </c>
-      <c r="N14" s="110" t="e">
+      <c r="N14" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O14" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6304,9 +6303,9 @@
       <c r="D15" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="108" t="str">
+      <c r="E15" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F15" s="109">
         <f>Report!$C$51</f>
@@ -6340,9 +6339,9 @@
         <f>IF(Report!G48&gt;=0,Report!G48,"")</f>
         <v/>
       </c>
-      <c r="N15" s="110" t="e">
+      <c r="N15" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.388888888891</v>
       </c>
       <c r="O15" t="str">
         <f>TRIM("Outfall: "&amp;Report!$C$52&amp;" "&amp;Report!$C$53&amp;" "&amp;Report!$C$54&amp;" "&amp;Report!$C$55)</f>
@@ -6366,9 +6365,9 @@
       <c r="D16" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="108" t="str">
+      <c r="E16" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F16" s="109">
         <f>Report!$J$51</f>
@@ -6402,9 +6401,9 @@
         <f>IF(Report!N35&gt;=0,Report!N35,"")</f>
         <v>1.0258692844512685</v>
       </c>
-      <c r="N16" s="110" t="e">
+      <c r="N16" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O16" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6428,9 +6427,9 @@
       <c r="D17" t="s">
         <v>75</v>
       </c>
-      <c r="E17" s="108" t="str">
+      <c r="E17" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F17" s="109">
         <f>Report!$J$51</f>
@@ -6464,9 +6463,9 @@
         <f>IF(Report!N36&gt;=0,Report!N36,"")</f>
         <v>0.96773318108499129</v>
       </c>
-      <c r="N17" s="110" t="e">
+      <c r="N17" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O17" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6490,9 +6489,9 @@
       <c r="D18" t="s">
         <v>75</v>
       </c>
-      <c r="E18" s="108" t="str">
+      <c r="E18" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F18" s="109">
         <f>Report!$J$51</f>
@@ -6526,9 +6525,9 @@
         <f>IF(Report!N37&gt;=0,Report!N37,"")</f>
         <v>1.002120290194243</v>
       </c>
-      <c r="N18" s="110" t="e">
+      <c r="N18" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O18" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6552,9 +6551,9 @@
       <c r="D19" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="108" t="str">
+      <c r="E19" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F19" s="109">
         <f>Report!$J$51</f>
@@ -6588,9 +6587,9 @@
         <f>IF(Report!N38&gt;=0,Report!N38,"")</f>
         <v>0.90990494312424308</v>
       </c>
-      <c r="N19" s="110" t="e">
+      <c r="N19" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O19" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6614,9 +6613,9 @@
       <c r="D20" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="108" t="str">
+      <c r="E20" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F20" s="109">
         <f>Report!$J$51</f>
@@ -6650,9 +6649,9 @@
         <f>IF(Report!N39&gt;=0,Report!N39,"")</f>
         <v>0.81259099330405993</v>
       </c>
-      <c r="N20" s="110" t="e">
+      <c r="N20" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O20" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6676,9 +6675,9 @@
       <c r="D21" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="108" t="str">
+      <c r="E21" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F21" s="109">
         <f>Report!$J$51</f>
@@ -6712,9 +6711,9 @@
         <f>IF(Report!N40&gt;=0,Report!N40,"")</f>
         <v>0.70788489234238416</v>
       </c>
-      <c r="N21" s="110" t="e">
+      <c r="N21" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O21" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6738,9 +6737,9 @@
       <c r="D22" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="108" t="str">
+      <c r="E22" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F22" s="109">
         <f>Report!$J$51</f>
@@ -6774,9 +6773,9 @@
         <f>IF(Report!N41&gt;=0,Report!N41,"")</f>
         <v>0.55111322265602558</v>
       </c>
-      <c r="N22" s="110" t="e">
+      <c r="N22" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O22" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6800,9 +6799,9 @@
       <c r="D23" t="s">
         <v>75</v>
       </c>
-      <c r="E23" s="108" t="str">
+      <c r="E23" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F23" s="109">
         <f>Report!$J$51</f>
@@ -6836,9 +6835,9 @@
         <f>IF(Report!N42&gt;=0,Report!N42,"")</f>
         <v>0.40512502239398046</v>
       </c>
-      <c r="N23" s="110" t="e">
+      <c r="N23" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O23" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6862,9 +6861,9 @@
       <c r="D24" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="108" t="str">
+      <c r="E24" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F24" s="109">
         <f>Report!$J$51</f>
@@ -6898,9 +6897,9 @@
         <f>IF(Report!N43&gt;=0,Report!N43,"")</f>
         <v>0.34007188011094763</v>
       </c>
-      <c r="N24" s="110" t="e">
+      <c r="N24" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O24" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6924,9 +6923,9 @@
       <c r="D25" t="s">
         <v>75</v>
       </c>
-      <c r="E25" s="108" t="str">
+      <c r="E25" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F25" s="109">
         <f>Report!$J$51</f>
@@ -6960,9 +6959,9 @@
         <f>IF(Report!N44&gt;=0,Report!N44,"")</f>
         <v>0.29109781586439698</v>
       </c>
-      <c r="N25" s="110" t="e">
+      <c r="N25" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O25" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -6986,9 +6985,9 @@
       <c r="D26" t="s">
         <v>75</v>
       </c>
-      <c r="E26" s="108" t="str">
+      <c r="E26" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F26" s="109">
         <f>Report!$J$51</f>
@@ -7022,9 +7021,9 @@
         <f>IF(Report!N45&gt;=0,Report!N45,"")</f>
         <v>0.27392756558864834</v>
       </c>
-      <c r="N26" s="110" t="e">
+      <c r="N26" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O26" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -7048,9 +7047,9 @@
       <c r="D27" t="s">
         <v>75</v>
       </c>
-      <c r="E27" s="108" t="str">
+      <c r="E27" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F27" s="109">
         <f>Report!$J$51</f>
@@ -7084,9 +7083,9 @@
         <f>IF(Report!N46&gt;=0,Report!N46,"")</f>
         <v>0.26453807399801049</v>
       </c>
-      <c r="N27" s="110" t="e">
+      <c r="N27" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O27" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -7110,9 +7109,9 @@
       <c r="D28" t="s">
         <v>75</v>
       </c>
-      <c r="E28" s="108" t="str">
+      <c r="E28" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F28" s="109">
         <f>Report!$J$51</f>
@@ -7146,9 +7145,9 @@
         <f>IF(Report!N47&gt;=0,Report!N47,"")</f>
         <v>0.23896294983841826</v>
       </c>
-      <c r="N28" s="110" t="e">
+      <c r="N28" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O28" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -7172,9 +7171,9 @@
       <c r="D29" t="s">
         <v>75</v>
       </c>
-      <c r="E29" s="108" t="str">
+      <c r="E29" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F29" s="109">
         <f>Report!$J$51</f>
@@ -7208,9 +7207,9 @@
         <f>IF(Report!N48&gt;=0,Report!N48,"")</f>
         <v/>
       </c>
-      <c r="N29" s="110" t="e">
+      <c r="N29" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O29" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -7234,9 +7233,9 @@
       <c r="D30" t="s">
         <v>75</v>
       </c>
-      <c r="E30" s="108" t="str">
+      <c r="E30" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F30" s="109">
         <f>Report!$J$51</f>
@@ -7270,9 +7269,9 @@
         <f>IF(Report!N49&gt;=0,Report!N49,"")</f>
         <v/>
       </c>
-      <c r="N30" s="110" t="e">
+      <c r="N30" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.398611111108</v>
       </c>
       <c r="O30" t="str">
         <f>TRIM("Hohm: "&amp;Report!$J$52&amp;" "&amp;Report!$J$53&amp;" "&amp;Report!$J$54&amp;" "&amp;Report!$J$55)</f>
@@ -7296,9 +7295,9 @@
       <c r="D31" t="s">
         <v>76</v>
       </c>
-      <c r="E31" s="108" t="str">
+      <c r="E31" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F31" s="109">
         <f>Report!$C$27</f>
@@ -7332,9 +7331,9 @@
         <f>IF(Report!N6&gt;=0,Report!N6,"")</f>
         <v>1.027917552726302</v>
       </c>
-      <c r="N31" s="110" t="e">
+      <c r="N31" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O31" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7358,9 +7357,9 @@
       <c r="D32" t="s">
         <v>76</v>
       </c>
-      <c r="E32" s="108" t="str">
+      <c r="E32" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F32" s="109">
         <f>Report!$C$27</f>
@@ -7394,9 +7393,9 @@
         <f>IF(Report!N7&gt;=0,Report!N7,"")</f>
         <v>1.0108768465503863</v>
       </c>
-      <c r="N32" s="110" t="e">
+      <c r="N32" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O32" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7420,9 +7419,9 @@
       <c r="D33" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="108" t="str">
+      <c r="E33" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F33" s="109">
         <f>Report!$C$27</f>
@@ -7456,9 +7455,9 @@
         <f>IF(Report!N8&gt;=0,Report!N8,"")</f>
         <v>1.0170120193615053</v>
       </c>
-      <c r="N33" s="110" t="e">
+      <c r="N33" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O33" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7482,9 +7481,9 @@
       <c r="D34" t="s">
         <v>76</v>
       </c>
-      <c r="E34" s="108" t="str">
+      <c r="E34" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F34" s="109">
         <f>Report!$C$27</f>
@@ -7518,9 +7517,9 @@
         <f>IF(Report!N9&gt;=0,Report!N9,"")</f>
         <v>0.96245832269451681</v>
       </c>
-      <c r="N34" s="110" t="e">
+      <c r="N34" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O34" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7544,9 +7543,9 @@
       <c r="D35" t="s">
         <v>76</v>
       </c>
-      <c r="E35" s="108" t="str">
+      <c r="E35" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F35" s="109">
         <f>Report!$C$27</f>
@@ -7580,9 +7579,9 @@
         <f>IF(Report!N10&gt;=0,Report!N10,"")</f>
         <v>0.91379179287841594</v>
       </c>
-      <c r="N35" s="110" t="e">
+      <c r="N35" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O35" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7606,9 +7605,9 @@
       <c r="D36" t="s">
         <v>76</v>
       </c>
-      <c r="E36" s="108" t="str">
+      <c r="E36" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F36" s="109">
         <f>Report!$C$27</f>
@@ -7642,9 +7641,9 @@
         <f>IF(Report!N11&gt;=0,Report!N11,"")</f>
         <v>0.50359064110835028</v>
       </c>
-      <c r="N36" s="110" t="e">
+      <c r="N36" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O36" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7668,9 +7667,9 @@
       <c r="D37" t="s">
         <v>76</v>
       </c>
-      <c r="E37" s="108" t="str">
+      <c r="E37" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F37" s="109">
         <f>Report!$C$27</f>
@@ -7704,9 +7703,9 @@
         <f>IF(Report!N12&gt;=0,Report!N12,"")</f>
         <v>0.40852662361273989</v>
       </c>
-      <c r="N37" s="110" t="e">
+      <c r="N37" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O37" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7730,9 +7729,9 @@
       <c r="D38" t="s">
         <v>76</v>
       </c>
-      <c r="E38" s="108" t="str">
+      <c r="E38" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F38" s="109">
         <f>Report!$C$27</f>
@@ -7766,9 +7765,9 @@
         <f>IF(Report!N13&gt;=0,Report!N13,"")</f>
         <v>0.37126132611262974</v>
       </c>
-      <c r="N38" s="110" t="e">
+      <c r="N38" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O38" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7792,9 +7791,9 @@
       <c r="D39" t="s">
         <v>76</v>
       </c>
-      <c r="E39" s="108" t="str">
+      <c r="E39" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F39" s="109">
         <f>Report!$C$27</f>
@@ -7828,9 +7827,9 @@
         <f>IF(Report!N14&gt;=0,Report!N14,"")</f>
         <v>0.33956431014063282</v>
       </c>
-      <c r="N39" s="110" t="e">
+      <c r="N39" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O39" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7854,9 +7853,9 @@
       <c r="D40" t="s">
         <v>76</v>
       </c>
-      <c r="E40" s="108" t="str">
+      <c r="E40" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F40" s="109">
         <f>Report!$C$27</f>
@@ -7890,9 +7889,9 @@
         <f>IF(Report!N15&gt;=0,Report!N15,"")</f>
         <v>0.3160887140211654</v>
       </c>
-      <c r="N40" s="110" t="e">
+      <c r="N40" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O40" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7916,9 +7915,9 @@
       <c r="D41" t="s">
         <v>76</v>
       </c>
-      <c r="E41" s="108" t="str">
+      <c r="E41" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F41" s="109">
         <f>Report!$C$27</f>
@@ -7952,9 +7951,9 @@
         <f>IF(Report!N16&gt;=0,Report!N16,"")</f>
         <v>0.30893648240638838</v>
       </c>
-      <c r="N41" s="110" t="e">
+      <c r="N41" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O41" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -7978,9 +7977,9 @@
       <c r="D42" t="s">
         <v>76</v>
       </c>
-      <c r="E42" s="108" t="str">
+      <c r="E42" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F42" s="109">
         <f>Report!$C$27</f>
@@ -8014,9 +8013,9 @@
         <f>IF(Report!N17&gt;=0,Report!N17,"")</f>
         <v>0.28488143978711639</v>
       </c>
-      <c r="N42" s="110" t="e">
+      <c r="N42" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O42" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8040,9 +8039,9 @@
       <c r="D43" t="s">
         <v>76</v>
       </c>
-      <c r="E43" s="108" t="str">
+      <c r="E43" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F43" s="109">
         <f>Report!$C$27</f>
@@ -8076,9 +8075,9 @@
         <f>IF(Report!N18&gt;=0,Report!N18,"")</f>
         <v>0.28236040201856555</v>
       </c>
-      <c r="N43" s="110" t="e">
+      <c r="N43" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O43" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8102,9 +8101,9 @@
       <c r="D44" t="s">
         <v>76</v>
       </c>
-      <c r="E44" s="108" t="str">
+      <c r="E44" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F44" s="109">
         <f>Report!$C$27</f>
@@ -8138,9 +8137,9 @@
         <f>IF(Report!N19&gt;=0,Report!N19,"")</f>
         <v>0.27171969104130284</v>
       </c>
-      <c r="N44" s="110" t="e">
+      <c r="N44" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O44" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8164,9 +8163,9 @@
       <c r="D45" t="s">
         <v>76</v>
       </c>
-      <c r="E45" s="108" t="str">
+      <c r="E45" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F45" s="109">
         <f>Report!$C$27</f>
@@ -8200,9 +8199,9 @@
         <f>IF(Report!N20&gt;=0,Report!N20,"")</f>
         <v/>
       </c>
-      <c r="N45" s="110" t="e">
+      <c r="N45" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O45" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8226,9 +8225,9 @@
       <c r="D46" t="s">
         <v>76</v>
       </c>
-      <c r="E46" s="108" t="str">
+      <c r="E46" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F46" s="109">
         <f>Report!$C$27</f>
@@ -8262,9 +8261,9 @@
         <f>IF(Report!N21&gt;=0,Report!N21,"")</f>
         <v/>
       </c>
-      <c r="N46" s="110" t="e">
+      <c r="N46" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O46" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8288,9 +8287,9 @@
       <c r="D47" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="108" t="str">
+      <c r="E47" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F47" s="109">
         <f>Report!$C$27</f>
@@ -8324,9 +8323,9 @@
         <f>IF(Report!N22&gt;=0,Report!N22,"")</f>
         <v/>
       </c>
-      <c r="N47" s="110" t="e">
+      <c r="N47" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.423611111109</v>
       </c>
       <c r="O47" t="str">
         <f>TRIM("Polly: "&amp;Report!$J$25&amp;" "&amp;Report!J$26&amp;" "&amp;Report!$J$27&amp;" "&amp;Report!$J$28)</f>
@@ -8350,9 +8349,9 @@
       <c r="D48" t="s">
         <v>77</v>
       </c>
-      <c r="E48" s="108" t="str">
+      <c r="E48" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F48" s="109">
         <f>Report!$J$24</f>
@@ -8386,9 +8385,9 @@
         <f>IF(Report!G6&gt;=0,Report!G6,"")</f>
         <v>1.0213202800387045</v>
       </c>
-      <c r="N48" s="110" t="e">
+      <c r="N48" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O48" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8412,9 +8411,9 @@
       <c r="D49" t="s">
         <v>77</v>
       </c>
-      <c r="E49" s="108" t="str">
+      <c r="E49" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F49" s="109">
         <f>Report!$J$24</f>
@@ -8448,9 +8447,9 @@
         <f>IF(Report!G7&gt;=0,Report!G7,"")</f>
         <v>1.0006511601854056</v>
       </c>
-      <c r="N49" s="110" t="e">
+      <c r="N49" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O49" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8474,9 +8473,9 @@
       <c r="D50" t="s">
         <v>77</v>
       </c>
-      <c r="E50" s="108" t="str">
+      <c r="E50" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F50" s="109">
         <f>Report!$J$24</f>
@@ -8510,9 +8509,9 @@
         <f>IF(Report!G8&gt;=0,Report!G8,"")</f>
         <v>1.0091745985536216</v>
       </c>
-      <c r="N50" s="110" t="e">
+      <c r="N50" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O50" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8536,9 +8535,9 @@
       <c r="D51" t="s">
         <v>77</v>
       </c>
-      <c r="E51" s="108" t="str">
+      <c r="E51" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F51" s="109">
         <f>Report!$J$24</f>
@@ -8572,9 +8571,9 @@
         <f>IF(Report!G9&gt;=0,Report!G9,"")</f>
         <v>1.0111405363623576</v>
       </c>
-      <c r="N51" s="110" t="e">
+      <c r="N51" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O51" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8598,9 +8597,9 @@
       <c r="D52" t="s">
         <v>77</v>
       </c>
-      <c r="E52" s="108" t="str">
+      <c r="E52" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F52" s="109">
         <f>Report!$J$24</f>
@@ -8634,9 +8633,9 @@
         <f>IF(Report!G10&gt;=0,Report!G10,"")</f>
         <v>0.92782704086296741</v>
       </c>
-      <c r="N52" s="110" t="e">
+      <c r="N52" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O52" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8660,9 +8659,9 @@
       <c r="D53" t="s">
         <v>77</v>
       </c>
-      <c r="E53" s="108" t="str">
+      <c r="E53" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F53" s="109">
         <f>Report!$J$24</f>
@@ -8696,9 +8695,9 @@
         <f>IF(Report!G11&gt;=0,Report!G11,"")</f>
         <v>0.72437215750674011</v>
       </c>
-      <c r="N53" s="110" t="e">
+      <c r="N53" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O53" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8722,9 +8721,9 @@
       <c r="D54" t="s">
         <v>77</v>
       </c>
-      <c r="E54" s="108" t="str">
+      <c r="E54" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F54" s="109">
         <f>Report!$J$24</f>
@@ -8758,9 +8757,9 @@
         <f>IF(Report!G12&gt;=0,Report!G12,"")</f>
         <v>0.54775199972342559</v>
       </c>
-      <c r="N54" s="110" t="e">
+      <c r="N54" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O54" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8784,9 +8783,9 @@
       <c r="D55" t="s">
         <v>77</v>
       </c>
-      <c r="E55" s="108" t="str">
+      <c r="E55" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F55" s="109">
         <f>Report!$J$24</f>
@@ -8820,9 +8819,9 @@
         <f>IF(Report!G13&gt;=0,Report!G13,"")</f>
         <v>0.45991314893382701</v>
       </c>
-      <c r="N55" s="110" t="e">
+      <c r="N55" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O55" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8846,9 +8845,9 @@
       <c r="D56" t="s">
         <v>77</v>
       </c>
-      <c r="E56" s="108" t="str">
+      <c r="E56" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F56" s="109">
         <f>Report!$J$24</f>
@@ -8882,9 +8881,9 @@
         <f>IF(Report!G14&gt;=0,Report!G14,"")</f>
         <v>0.40137416709379803</v>
       </c>
-      <c r="N56" s="110" t="e">
+      <c r="N56" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O56" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8908,9 +8907,9 @@
       <c r="D57" t="s">
         <v>77</v>
       </c>
-      <c r="E57" s="108" t="str">
+      <c r="E57" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F57" s="109">
         <f>Report!$J$24</f>
@@ -8944,9 +8943,9 @@
         <f>IF(Report!G15&gt;=0,Report!G15,"")</f>
         <v>0.3743187967225306</v>
       </c>
-      <c r="N57" s="110" t="e">
+      <c r="N57" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O57" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -8970,9 +8969,9 @@
       <c r="D58" t="s">
         <v>77</v>
       </c>
-      <c r="E58" s="108" t="str">
+      <c r="E58" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F58" s="109">
         <f>Report!$J$24</f>
@@ -9006,9 +9005,9 @@
         <f>IF(Report!G16&gt;=0,Report!G16,"")</f>
         <v>0.3582878646791286</v>
       </c>
-      <c r="N58" s="110" t="e">
+      <c r="N58" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O58" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9032,9 +9031,9 @@
       <c r="D59" t="s">
         <v>77</v>
       </c>
-      <c r="E59" s="108" t="str">
+      <c r="E59" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F59" s="109">
         <f>Report!$J$24</f>
@@ -9068,9 +9067,9 @@
         <f>IF(Report!G17&gt;=0,Report!G17,"")</f>
         <v>0.33550757358072325</v>
       </c>
-      <c r="N59" s="110" t="e">
+      <c r="N59" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O59" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9094,9 +9093,9 @@
       <c r="D60" t="s">
         <v>77</v>
       </c>
-      <c r="E60" s="108" t="str">
+      <c r="E60" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F60" s="109">
         <f>Report!$J$24</f>
@@ -9130,9 +9129,9 @@
         <f>IF(Report!G18&gt;=0,Report!G18,"")</f>
         <v>0.32868987156509827</v>
       </c>
-      <c r="N60" s="110" t="e">
+      <c r="N60" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O60" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9156,9 +9155,9 @@
       <c r="D61" t="s">
         <v>77</v>
       </c>
-      <c r="E61" s="108" t="str">
+      <c r="E61" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F61" s="109">
         <f>Report!$J$24</f>
@@ -9192,9 +9191,9 @@
         <f>IF(Report!G19&gt;=0,Report!G19,"")</f>
         <v>0.33189626932874633</v>
       </c>
-      <c r="N61" s="110" t="e">
+      <c r="N61" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O61" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9218,9 +9217,9 @@
       <c r="D62" t="s">
         <v>77</v>
       </c>
-      <c r="E62" s="108" t="str">
+      <c r="E62" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F62" s="109">
         <f>Report!$J$24</f>
@@ -9254,9 +9253,9 @@
         <f>IF(Report!G20&gt;=0,Report!G20,"")</f>
         <v>0.30030036511448049</v>
       </c>
-      <c r="N62" s="110" t="e">
+      <c r="N62" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O62" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9280,9 +9279,9 @@
       <c r="D63" t="s">
         <v>77</v>
       </c>
-      <c r="E63" s="108" t="str">
+      <c r="E63" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F63" s="109">
         <f>Report!$J$24</f>
@@ -9316,9 +9315,9 @@
         <f>IF(Report!G21&gt;=0,Report!G21,"")</f>
         <v>0.28656200578592095</v>
       </c>
-      <c r="N63" s="110" t="e">
+      <c r="N63" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O63" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9342,9 +9341,9 @@
       <c r="D64" t="s">
         <v>77</v>
       </c>
-      <c r="E64" s="108" t="str">
+      <c r="E64" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F64" s="109">
         <f>Report!$J$24</f>
@@ -9378,9 +9377,9 @@
         <f>IF(Report!G22&gt;=0,Report!G22,"")</f>
         <v>0.27654163510981783</v>
       </c>
-      <c r="N64" s="110" t="e">
+      <c r="N64" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O64" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9404,9 +9403,9 @@
       <c r="D65" t="s">
         <v>77</v>
       </c>
-      <c r="E65" s="108" t="str">
+      <c r="E65" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F65" s="109">
         <f>Report!$J$24</f>
@@ -9440,9 +9439,9 @@
         <f>IF(Report!G23&gt;=0,Report!G23,"")</f>
         <v>0.26125984798706958</v>
       </c>
-      <c r="N65" s="110" t="e">
+      <c r="N65" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O65" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9466,9 +9465,9 @@
       <c r="D66" t="s">
         <v>77</v>
       </c>
-      <c r="E66" s="108" t="str">
+      <c r="E66" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F66" s="109">
         <f>Report!$J$24</f>
@@ -9502,9 +9501,9 @@
         <f>IF(Report!G24&gt;=0,Report!G24,"")</f>
         <v>0.23636326229881302</v>
       </c>
-      <c r="N66" s="110" t="e">
+      <c r="N66" s="110">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O66" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9528,9 +9527,9 @@
       <c r="D67" t="s">
         <v>77</v>
       </c>
-      <c r="E67" s="108" t="str">
+      <c r="E67" s="108">
         <f>Report!$B$2</f>
-        <v>23/9/2026</v>
+        <v>46288</v>
       </c>
       <c r="F67" s="109">
         <f>Report!$J$24</f>
@@ -9564,9 +9563,9 @@
         <f>IF(Report!G25&gt;=0,Report!G25,"")</f>
         <v>0.21976589330221175</v>
       </c>
-      <c r="N67" s="110" t="e">
+      <c r="N67" s="110">
         <f t="shared" ref="N67" si="1">E67+F67</f>
-        <v>#VALUE!</v>
+        <v>46288.40902777778</v>
       </c>
       <c r="O67" t="str">
         <f>TRIM("5KM: "&amp;Report!$C$28&amp;" "&amp;Report!$C$29&amp;" "&amp;Report!$C$30&amp;" "&amp;Report!$C$31)</f>
@@ -9641,6 +9640,9 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
+  </headerFooter>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -12756,6 +12758,8 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0.25" top="1" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="89" orientation="portrait" horizontalDpi="1200" r:id="rId1"/>
-  <headerFooter alignWithMargins="0"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>